<commit_message>
add footer link 58b517ad6e1249405b4a130345737ec14cafa087
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-patient.xlsx
+++ b/main/ig/StructureDefinition-fr-patient.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-05T08:22:23+00:00</t>
+    <t>2025-09-26T14:20:13+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -75,7 +75,7 @@
     <t>Interop'Santé (http://interopsante.org/)</t>
   </si>
   <si>
-    <t>InteropSanté (fhir@interopsante.org(work))</t>
+    <t>InteropSanté (fhir@interopsante.org(Work))</t>
   </si>
   <si>
     <t>Jurisdiction</t>
@@ -374,7 +374,7 @@
     <t>A human language.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/languages</t>
+    <t>http://hl7.org/fhir/ValueSet/languages|4.0.1</t>
   </si>
   <si>
     <t>Resource.language</t>
@@ -732,7 +732,7 @@
     <t>The domestic partnership status of a person.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/marital-status</t>
+    <t>http://hl7.org/fhir/ValueSet/marital-status|4.0.1</t>
   </si>
   <si>
     <t>player[classCode=PSN]/maritalStatusCode</t>
@@ -880,7 +880,7 @@
     <t>The nature of the relationship between a patient and a contact person for that patient.</t>
   </si>
   <si>
-    <t>http://hl7.org/fhir/ValueSet/patient-contactrelationship</t>
+    <t>http://hl7.org/fhir/ValueSet/patient-contactrelationship|4.0.1</t>
   </si>
   <si>
     <t>code</t>
@@ -949,7 +949,7 @@
     <t>Patient.contact.organization</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Organization)
+    <t xml:space="preserve">Reference(Organization|4.0.1)
 </t>
   </si>
   <si>
@@ -1073,7 +1073,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Organization|Practitioner|PractitionerRole)
+    <t xml:space="preserve">Reference(Organization|4.0.1|Practitioner|4.0.1|PractitionerRole|4.0.1)
 </t>
   </si>
   <si>
@@ -1144,7 +1144,7 @@
     <t>Patient.link.other</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Patient|RelatedPerson)
+    <t xml:space="preserve">Reference(Patient|4.0.1|RelatedPerson|4.0.1)
 </t>
   </si>
   <si>
@@ -1510,7 +1510,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="42.9296875" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="56.515625" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>
@@ -1525,7 +1525,7 @@
     <col min="23" max="23" width="16.3203125" customWidth="true" bestFit="true"/>
     <col min="24" max="24" width="16.16796875" customWidth="true" bestFit="true"/>
     <col min="25" max="25" width="69.35546875" customWidth="true" bestFit="true"/>
-    <col min="26" max="26" width="44.51171875" customWidth="true" bestFit="true"/>
+    <col min="26" max="26" width="48.33203125" customWidth="true" bestFit="true"/>
     <col min="27" max="27" width="5.44140625" customWidth="true" bestFit="true"/>
     <col min="28" max="28" width="19.4765625" customWidth="true" bestFit="true"/>
     <col min="29" max="29" width="17.65625" customWidth="true" bestFit="true"/>

</xml_diff>

<commit_message>
Update GitHub Actions workflow for CI-build 5b1dd34aadf1e9db532915a0303f62755a9999f7
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-fr-patient.xlsx
+++ b/main/ig/StructureDefinition-fr-patient.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-09-26T14:20:13+00:00</t>
+    <t>2026-06-29T09:18:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -2718,7 +2718,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="11" hidden="true">
+    <row r="11">
       <c r="A11" t="s" s="2">
         <v>147</v>
       </c>
@@ -6962,12 +6962,12 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AO46">
-    <filterColumn colId="6">
+    <filterColumn colId="7">
       <customFilters>
         <customFilter operator="notEqual" val=" "/>
       </customFilters>
     </filterColumn>
-    <filterColumn colId="26">
+    <filterColumn colId="27">
       <filters blank="true"/>
     </filterColumn>
   </autoFilter>

</xml_diff>